<commit_message>
completed responses for assignment 3
</commit_message>
<xml_diff>
--- a/02_activities/assignments/assignment_3_files/Dataset_2:Overnight_Spending_by_Overseas_Visitors.xlsx
+++ b/02_activities/assignments/assignment_3_files/Dataset_2:Overnight_Spending_by_Overseas_Visitors.xlsx
@@ -5,53 +5,17 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/charissachan/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/charissachan/Desktop/DSI/visualization/02_activities/assignments/assignment_3_files/Dataset_2:"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F1788BA-295E-A448-BA75-5FF674746853}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18A20566-641A-5D4D-A9B1-45A7FB89E3BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3840" yWindow="1060" windowWidth="31980" windowHeight="19700" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3840" yWindow="740" windowWidth="31980" windowHeight="19700" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Visualization 2" sheetId="3" r:id="rId1"/>
     <sheet name="1990-2021" sheetId="1" r:id="rId2"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlchart.v1.0" hidden="1">'1990-2021'!$A$1:$A$3</definedName>
-    <definedName name="_xlchart.v1.1" hidden="1">'1990-2021'!$A$4:$A$31</definedName>
-    <definedName name="_xlchart.v1.10" hidden="1">'1990-2021'!$F$1:$F$3</definedName>
-    <definedName name="_xlchart.v1.11" hidden="1">'1990-2021'!$F$4:$F$31</definedName>
-    <definedName name="_xlchart.v1.12" hidden="1">'1990-2021'!$G$1:$G$3</definedName>
-    <definedName name="_xlchart.v1.13" hidden="1">'1990-2021'!$G$4:$G$31</definedName>
-    <definedName name="_xlchart.v1.14" hidden="1">'1990-2021'!$H$1:$H$3</definedName>
-    <definedName name="_xlchart.v1.15" hidden="1">'1990-2021'!$H$4:$H$31</definedName>
-    <definedName name="_xlchart.v1.16" hidden="1">'1990-2021'!$I$1:$I$3</definedName>
-    <definedName name="_xlchart.v1.17" hidden="1">'1990-2021'!$I$4:$I$31</definedName>
-    <definedName name="_xlchart.v1.18" hidden="1">'1990-2021'!$J$1:$J$3</definedName>
-    <definedName name="_xlchart.v1.19" hidden="1">'1990-2021'!$J$4:$J$31</definedName>
-    <definedName name="_xlchart.v1.2" hidden="1">'1990-2021'!$B$1:$B$3</definedName>
-    <definedName name="_xlchart.v1.20" hidden="1">'1990-2021'!$K$1:$K$3</definedName>
-    <definedName name="_xlchart.v1.21" hidden="1">'1990-2021'!$K$4:$K$31</definedName>
-    <definedName name="_xlchart.v1.22" hidden="1">'1990-2021'!$L$1:$L$3</definedName>
-    <definedName name="_xlchart.v1.23" hidden="1">'1990-2021'!$L$4:$L$31</definedName>
-    <definedName name="_xlchart.v1.24" hidden="1">'1990-2021'!$M$1:$M$3</definedName>
-    <definedName name="_xlchart.v1.25" hidden="1">'1990-2021'!$M$4:$M$31</definedName>
-    <definedName name="_xlchart.v1.26" hidden="1">'1990-2021'!$N$1:$N$3</definedName>
-    <definedName name="_xlchart.v1.27" hidden="1">'1990-2021'!$N$4:$N$31</definedName>
-    <definedName name="_xlchart.v1.28" hidden="1">'1990-2021'!$O$1:$O$3</definedName>
-    <definedName name="_xlchart.v1.29" hidden="1">'1990-2021'!$O$4:$O$31</definedName>
-    <definedName name="_xlchart.v1.3" hidden="1">'1990-2021'!$B$4:$B$31</definedName>
-    <definedName name="_xlchart.v1.30" hidden="1">'1990-2021'!$P$1:$P$3</definedName>
-    <definedName name="_xlchart.v1.31" hidden="1">'1990-2021'!$P$4:$P$31</definedName>
-    <definedName name="_xlchart.v1.32" hidden="1">'1990-2021'!$Q$1:$Q$3</definedName>
-    <definedName name="_xlchart.v1.33" hidden="1">'1990-2021'!$Q$4:$Q$31</definedName>
-    <definedName name="_xlchart.v1.4" hidden="1">'1990-2021'!$C$1:$C$3</definedName>
-    <definedName name="_xlchart.v1.5" hidden="1">'1990-2021'!$C$4:$C$31</definedName>
-    <definedName name="_xlchart.v1.6" hidden="1">'1990-2021'!$D$1:$D$3</definedName>
-    <definedName name="_xlchart.v1.7" hidden="1">'1990-2021'!$D$4:$D$31</definedName>
-    <definedName name="_xlchart.v1.8" hidden="1">'1990-2021'!$E$1:$E$3</definedName>
-    <definedName name="_xlchart.v1.9" hidden="1">'1990-2021'!$E$4:$E$31</definedName>
-  </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
@@ -1886,13 +1850,100 @@
             <c:symbol val="none"/>
           </c:marker>
           <c:val>
-            <c:numLit>
-              <c:formatCode>General</c:formatCode>
-              <c:ptCount val="1"/>
-              <c:pt idx="0">
-                <c:v>1</c:v>
-              </c:pt>
-            </c:numLit>
+            <c:numRef>
+              <c:f>'1990-2021'!$L$3:$L$31</c:f>
+              <c:numCache>
+                <c:formatCode>#,##0.0</c:formatCode>
+                <c:ptCount val="29"/>
+                <c:pt idx="0" formatCode="General">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>17.8537</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>10.321899999999999</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>10.9604</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>16.261299999999999</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>16.981999999999999</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>19.7395</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>48.739699999999999</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>88.1982</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>60.247500000000002</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>61.833399999999997</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>64.400000000000006</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>62.8</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>73.5</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>50.9</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>32.5</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>85.1</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>185.4</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>183.8</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>157.6</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>129.69999999999999</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>211.2</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>268.2</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>326.3</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>337.7</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>574.6</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>589</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>758.3</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>842.2</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
           </c:val>
           <c:smooth val="0"/>
           <c:extLst>

</xml_diff>